<commit_message>
SID STAR database load now loading correctly SID STAR waypoints in WayPoints database
</commit_message>
<xml_diff>
--- a/Airlines-Services/trajectory/management/commands/SidStar/SID-LIBD-07-PISIP.xlsx
+++ b/Airlines-Services/trajectory/management/commands/SidStar/SID-LIBD-07-PISIP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\git\Airlines-Services\Airlines-Services\trajectory\management\commands\SidStar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0BA08B-4C54-48A3-911A-FC12998EED0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1709EE27-5BCF-4920-BB9F-DE7941BEBAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5900" yWindow="3360" windowWidth="15510" windowHeight="11170" xr2:uid="{5B8640E8-34B0-4460-913B-4CC43B5210E1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{5B8640E8-34B0-4460-913B-4CC43B5210E1}"/>
   </bookViews>
   <sheets>
     <sheet name="WayPoints" sheetId="1" r:id="rId1"/>
@@ -143,31 +143,31 @@
     <t>E016°32'57.70"</t>
   </si>
   <si>
-    <t>RWY-07-001</t>
-  </si>
-  <si>
-    <t>RWY-07-002</t>
-  </si>
-  <si>
-    <t>RWY-07-003</t>
-  </si>
-  <si>
-    <t>RWY-07-004</t>
-  </si>
-  <si>
-    <t>RWY-07-005</t>
-  </si>
-  <si>
-    <t>RWY-07-006</t>
-  </si>
-  <si>
-    <t>RWY-07-007</t>
-  </si>
-  <si>
     <t>N41°01'33.00"</t>
   </si>
   <si>
     <t>E016°40'07.00"</t>
+  </si>
+  <si>
+    <t>RWY_07_001</t>
+  </si>
+  <si>
+    <t>RWY_07_002</t>
+  </si>
+  <si>
+    <t>RWY_07_003</t>
+  </si>
+  <si>
+    <t>RWY_07_004</t>
+  </si>
+  <si>
+    <t>RWY_07_005</t>
+  </si>
+  <si>
+    <t>RWY_07_006</t>
+  </si>
+  <si>
+    <t>RWY_07_007</t>
   </si>
 </sst>
 </file>
@@ -606,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -629,7 +629,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
@@ -652,7 +652,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
         <v>16</v>
@@ -675,7 +675,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -698,7 +698,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
         <v>22</v>
@@ -721,13 +721,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
         <v>1</v>
@@ -744,7 +744,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>26</v>

</xml_diff>